<commit_message>
add: main evaluation comparison
</commit_message>
<xml_diff>
--- a/analysis/summary_doctor_models.xlsx
+++ b/analysis/summary_doctor_models.xlsx
@@ -838,6 +838,9 @@
       <c r="R6" s="1" t="n">
         <v>0.1</v>
       </c>
+      <c r="S6" s="1" t="n">
+        <v>0.7733</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1075,6 +1078,15 @@
       <c r="D6" s="2" t="n">
         <v>230</v>
       </c>
+      <c r="E6" s="2" t="n">
+        <v>217</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>221</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">

</xml_diff>